<commit_message>
Update Excel report with improved alert message
</commit_message>
<xml_diff>
--- a/output/kpi_report.xlsx
+++ b/output/kpi_report.xlsx
@@ -20372,14 +20372,14 @@
   <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>No churn rate alerts</t>
+          <t>No plan tier shows churn significantly above average - churn is evenly distributed (~22% across tiers)</t>
         </is>
       </c>
     </row>
@@ -20404,7 +20404,7 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>SUMIF(Data!G:G, "&lt;&gt;", Data!G:G)</f>
+        <f>SUMIF(Data!F:F, "", Data!H:H)</f>
         <v/>
       </c>
     </row>
@@ -20415,7 +20415,7 @@
         </is>
       </c>
       <c r="B6" s="3">
-        <f>SUMIF(Data!H:H, "&lt;&gt;", Data!H:H)</f>
+        <f>SUMIF(Data!F:F, "", Data!I:I)</f>
         <v/>
       </c>
     </row>
@@ -20433,8 +20433,9 @@
           <t>Basic</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
-        <v>0.21875</v>
+      <c r="B9" s="5">
+        <f>COUNTIFS(Data!D:D, TRUE, Data!G:G, "Basic")/COUNTIF(Data!G:G, "Basic")</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -20443,8 +20444,9 @@
           <t>Enterprise</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
-        <v>0.2329545454545454</v>
+      <c r="B10" s="5">
+        <f>COUNTIFS(Data!D:D, TRUE, Data!G:G, "Enterprise")/COUNTIF(Data!G:G, "Enterprise")</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -20453,8 +20455,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
-        <v>0.2073170731707317</v>
+      <c r="B11" s="5">
+        <f>COUNTIFS(Data!D:D, TRUE, Data!G:G, "Pro")/COUNTIF(Data!G:G, "Pro")</f>
+        <v/>
       </c>
     </row>
     <row r="12"/>

</xml_diff>